<commit_message>
Clean in/out columns: set to 'OFF' and remove template yellow fill for off/standby days
</commit_message>
<xml_diff>
--- a/Attendance_2026_10_25.xlsx
+++ b/Attendance_2026_10_25.xlsx
@@ -16,11 +16,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="_-* #,##0.00\ &quot;ل.س.‏&quot;_-;\-* #,##0.00\ &quot;ل.س.‏&quot;_-;_-* &quot;-&quot;??\ &quot;ل.س.‏&quot;_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="hh:mm"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="hh:mm"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ &quot;ل.س.‏&quot;_-;\-* #,##0.00\ &quot;ل.س.‏&quot;_-;_-* &quot;-&quot;??\ &quot;ل.س.‏&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -111,6 +111,11 @@
       <color rgb="FFFF0000"/>
       <sz val="16"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -190,9 +195,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -242,14 +247,23 @@
     <xf numFmtId="20" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -681,13 +695,13 @@
           <t>Omar Elnemr</t>
         </is>
       </c>
-      <c r="C2" s="17" t="n">
+      <c r="C2" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D2" s="18" t="n">
+      <c r="D2" s="21" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="E2" s="18" t="n">
+      <c r="E2" s="21" t="n">
         <v>0.1319444444444444</v>
       </c>
       <c r="F2" s="7" t="n"/>
@@ -717,13 +731,13 @@
           <t>Mohammad Almohammad</t>
         </is>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D3" s="18" t="n">
+      <c r="D3" s="21" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="21" t="n">
         <v>0.8055555555555556</v>
       </c>
       <c r="F3" s="8" t="n"/>
@@ -753,13 +767,13 @@
           <t>Hanan Tinawi</t>
         </is>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="21" t="n">
         <v>0.8333333333333334</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="21" t="n">
         <v>0.125</v>
       </c>
       <c r="F4" s="8" t="n"/>
@@ -789,14 +803,18 @@
           <t>Osama Alkabbani</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D5" s="16" t="n">
-        <v>0.3541666666666667</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>0.6875</v>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
       </c>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="8" t="n"/>
@@ -825,14 +843,18 @@
           <t>Yasmin Tatary</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D6" s="16" t="n">
-        <v>0.3541666666666667</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>0.6875</v>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
       </c>
       <c r="F6" s="8" t="n"/>
       <c r="G6" s="8" t="n"/>
@@ -861,14 +883,18 @@
           <t>Joudi Alghorani</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D7" s="16" t="n">
-        <v>0.3541666666666667</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>0.6875</v>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
       </c>
       <c r="F7" s="8" t="n"/>
       <c r="G7" s="8" t="n"/>
@@ -897,13 +923,13 @@
           <t>Khaled Mohammad Mlas</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="21" t="n">
         <v>0.8298611111111112</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="21" t="n">
         <v>0.09722222222222222</v>
       </c>
       <c r="F8" s="8" t="n"/>
@@ -933,14 +959,18 @@
           <t>Raboushee</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D9" s="16" t="n">
-        <v>0.3541666666666667</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>0.6875</v>
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
       </c>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="8" t="n"/>
@@ -969,13 +999,13 @@
           <t>Rasheed Akel</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="20" t="n">
         <v>46320</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="21" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="21" t="n">
         <v>0.8055555555555556</v>
       </c>
       <c r="F10" s="8" t="n"/>

</xml_diff>